<commit_message>
nuevo excel, nuevas instrucciones, revision del 9 de marzo del 2026
</commit_message>
<xml_diff>
--- a/datos/datos_calidad_aire_DIARIO.xlsx
+++ b/datos/datos_calidad_aire_DIARIO.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -73,7 +73,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -81,23 +81,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -596,1362 +587,1362 @@
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_AGUA SANTA</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_AGUA SANTA</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_AGUA SANTA</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_AGUA SANTA</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_AGUA SANTA</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_AGUA SANTA</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_AGUA SANTA</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_AGUA SANTA</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_AGUA SANTA</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_AGUA SANTA</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_AGUA SANTA</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_AGUA SANTA</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_ATLIXCO</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_ATLIXCO</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_ATLIXCO</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_ATLIXCO</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_ATLIXCO</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_ATLIXCO</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_ATLIXCO</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_ATLIXCO</t>
         </is>
       </c>
-      <c r="V1" s="3" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_ATLIXCO</t>
         </is>
       </c>
-      <c r="W1" s="3" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_ATLIXCO</t>
         </is>
       </c>
-      <c r="X1" s="3" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_ATLIXCO</t>
         </is>
       </c>
-      <c r="Y1" s="3" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_ATLIXCO</t>
         </is>
       </c>
-      <c r="Z1" s="3" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_BINE</t>
         </is>
       </c>
-      <c r="AA1" s="3" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_BINE</t>
         </is>
       </c>
-      <c r="AB1" s="3" t="inlineStr">
+      <c r="AB1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_BINE</t>
         </is>
       </c>
-      <c r="AC1" s="3" t="inlineStr">
+      <c r="AC1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_BINE</t>
         </is>
       </c>
-      <c r="AD1" s="3" t="inlineStr">
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_BINE</t>
         </is>
       </c>
-      <c r="AE1" s="3" t="inlineStr">
+      <c r="AE1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_BINE</t>
         </is>
       </c>
-      <c r="AF1" s="3" t="inlineStr">
+      <c r="AF1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_BINE</t>
         </is>
       </c>
-      <c r="AG1" s="3" t="inlineStr">
+      <c r="AG1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_BINE</t>
         </is>
       </c>
-      <c r="AH1" s="3" t="inlineStr">
+      <c r="AH1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_BINE</t>
         </is>
       </c>
-      <c r="AI1" s="3" t="inlineStr">
+      <c r="AI1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_BINE</t>
         </is>
       </c>
-      <c r="AJ1" s="3" t="inlineStr">
+      <c r="AJ1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_BINE</t>
         </is>
       </c>
-      <c r="AK1" s="3" t="inlineStr">
+      <c r="AK1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_BINE</t>
         </is>
       </c>
-      <c r="AL1" s="3" t="inlineStr">
+      <c r="AL1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_NINFAS</t>
         </is>
       </c>
-      <c r="AM1" s="3" t="inlineStr">
+      <c r="AM1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_NINFAS</t>
         </is>
       </c>
-      <c r="AN1" s="3" t="inlineStr">
+      <c r="AN1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_NINFAS</t>
         </is>
       </c>
-      <c r="AO1" s="3" t="inlineStr">
+      <c r="AO1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_NINFAS</t>
         </is>
       </c>
-      <c r="AP1" s="3" t="inlineStr">
+      <c r="AP1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_NINFAS</t>
         </is>
       </c>
-      <c r="AQ1" s="3" t="inlineStr">
+      <c r="AQ1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_NINFAS</t>
         </is>
       </c>
-      <c r="AR1" s="3" t="inlineStr">
+      <c r="AR1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_NINFAS</t>
         </is>
       </c>
-      <c r="AS1" s="3" t="inlineStr">
+      <c r="AS1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_NINFAS</t>
         </is>
       </c>
-      <c r="AT1" s="3" t="inlineStr">
+      <c r="AT1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_NINFAS</t>
         </is>
       </c>
-      <c r="AU1" s="3" t="inlineStr">
+      <c r="AU1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_NINFAS</t>
         </is>
       </c>
-      <c r="AV1" s="3" t="inlineStr">
+      <c r="AV1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_NINFAS</t>
         </is>
       </c>
-      <c r="AW1" s="3" t="inlineStr">
+      <c r="AW1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_NINFAS</t>
         </is>
       </c>
-      <c r="AX1" s="3" t="inlineStr">
+      <c r="AX1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_TEHUACAN</t>
         </is>
       </c>
-      <c r="AY1" s="3" t="inlineStr">
+      <c r="AY1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_TEHUACAN</t>
         </is>
       </c>
-      <c r="AZ1" s="3" t="inlineStr">
+      <c r="AZ1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_TEHUACAN</t>
         </is>
       </c>
-      <c r="BA1" s="3" t="inlineStr">
+      <c r="BA1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_TEHUACAN</t>
         </is>
       </c>
-      <c r="BB1" s="3" t="inlineStr">
+      <c r="BB1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_TEHUACAN</t>
         </is>
       </c>
-      <c r="BC1" s="3" t="inlineStr">
+      <c r="BC1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_TEHUACAN</t>
         </is>
       </c>
-      <c r="BD1" s="3" t="inlineStr">
+      <c r="BD1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_TEHUACAN</t>
         </is>
       </c>
-      <c r="BE1" s="3" t="inlineStr">
+      <c r="BE1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_TEHUACAN</t>
         </is>
       </c>
-      <c r="BF1" s="3" t="inlineStr">
+      <c r="BF1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_TEHUACAN</t>
         </is>
       </c>
-      <c r="BG1" s="3" t="inlineStr">
+      <c r="BG1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_TEHUACAN</t>
         </is>
       </c>
-      <c r="BH1" s="3" t="inlineStr">
+      <c r="BH1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_TEHUACAN</t>
         </is>
       </c>
-      <c r="BI1" s="3" t="inlineStr">
+      <c r="BI1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_TEHUACAN</t>
         </is>
       </c>
-      <c r="BJ1" s="3" t="inlineStr">
+      <c r="BJ1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BK1" s="3" t="inlineStr">
+      <c r="BK1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BL1" s="3" t="inlineStr">
+      <c r="BL1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BM1" s="3" t="inlineStr">
+      <c r="BM1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BN1" s="3" t="inlineStr">
+      <c r="BN1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BO1" s="3" t="inlineStr">
+      <c r="BO1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BP1" s="3" t="inlineStr">
+      <c r="BP1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BQ1" s="3" t="inlineStr">
+      <c r="BQ1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BR1" s="3" t="inlineStr">
+      <c r="BR1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BS1" s="3" t="inlineStr">
+      <c r="BS1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BT1" s="3" t="inlineStr">
+      <c r="BT1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BU1" s="3" t="inlineStr">
+      <c r="BU1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BV1" s="3" t="inlineStr">
+      <c r="BV1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_UTP</t>
         </is>
       </c>
-      <c r="BW1" s="3" t="inlineStr">
+      <c r="BW1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_UTP</t>
         </is>
       </c>
-      <c r="BX1" s="3" t="inlineStr">
+      <c r="BX1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_UTP</t>
         </is>
       </c>
-      <c r="BY1" s="3" t="inlineStr">
+      <c r="BY1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_UTP</t>
         </is>
       </c>
-      <c r="BZ1" s="3" t="inlineStr">
+      <c r="BZ1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_UTP</t>
         </is>
       </c>
-      <c r="CA1" s="3" t="inlineStr">
+      <c r="CA1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_UTP</t>
         </is>
       </c>
-      <c r="CB1" s="3" t="inlineStr">
+      <c r="CB1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_UTP</t>
         </is>
       </c>
-      <c r="CC1" s="3" t="inlineStr">
+      <c r="CC1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_UTP</t>
         </is>
       </c>
-      <c r="CD1" s="3" t="inlineStr">
+      <c r="CD1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_UTP</t>
         </is>
       </c>
-      <c r="CE1" s="3" t="inlineStr">
+      <c r="CE1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_UTP</t>
         </is>
       </c>
-      <c r="CF1" s="3" t="inlineStr">
+      <c r="CF1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_UTP</t>
         </is>
       </c>
-      <c r="CG1" s="3" t="inlineStr">
+      <c r="CG1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_UTP</t>
         </is>
       </c>
-      <c r="CH1" s="3" t="inlineStr">
+      <c r="CH1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_VELODROMO</t>
         </is>
       </c>
-      <c r="CI1" s="3" t="inlineStr">
+      <c r="CI1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_VELODROMO</t>
         </is>
       </c>
-      <c r="CJ1" s="3" t="inlineStr">
+      <c r="CJ1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_VELODROMO</t>
         </is>
       </c>
-      <c r="CK1" s="3" t="inlineStr">
+      <c r="CK1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_VELODROMO</t>
         </is>
       </c>
-      <c r="CL1" s="3" t="inlineStr">
+      <c r="CL1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_VELODROMO</t>
         </is>
       </c>
-      <c r="CM1" s="3" t="inlineStr">
+      <c r="CM1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_VELODROMO</t>
         </is>
       </c>
-      <c r="CN1" s="3" t="inlineStr">
+      <c r="CN1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_VELODROMO</t>
         </is>
       </c>
-      <c r="CO1" s="3" t="inlineStr">
+      <c r="CO1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_VELODROMO</t>
         </is>
       </c>
-      <c r="CP1" s="3" t="inlineStr">
+      <c r="CP1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_VELODROMO</t>
         </is>
       </c>
-      <c r="CQ1" s="3" t="inlineStr">
+      <c r="CQ1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_VELODROMO</t>
         </is>
       </c>
-      <c r="CR1" s="3" t="inlineStr">
+      <c r="CR1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_VELODROMO</t>
         </is>
       </c>
-      <c r="CS1" s="3" t="inlineStr">
+      <c r="CS1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_VELODROMO</t>
         </is>
       </c>
-      <c r="CT1" s="3" t="inlineStr">
+      <c r="CT1" s="2" t="inlineStr">
         <is>
           <t>Calidad del aire</t>
         </is>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="4" t="n">
+      <c r="A2" s="3" t="n">
         <v>46054</v>
       </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="n">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
         <v>0.057</v>
       </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="n">
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n">
         <v>0.019</v>
       </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="n">
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="n">
         <v>0.51</v>
       </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="n">
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="n">
         <v>0.001</v>
       </c>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K2" s="8" t="n">
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="K2" s="7" t="n">
         <v>27</v>
       </c>
-      <c r="L2" s="9" t="inlineStr">
+      <c r="L2" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="M2" s="8" t="n">
+      <c r="M2" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="N2" s="10" t="inlineStr"/>
-      <c r="O2" s="10" t="inlineStr"/>
-      <c r="P2" s="10" t="inlineStr"/>
-      <c r="Q2" s="10" t="inlineStr"/>
-      <c r="R2" s="10" t="inlineStr"/>
-      <c r="S2" s="10" t="inlineStr"/>
-      <c r="T2" s="10" t="inlineStr"/>
-      <c r="U2" s="10" t="inlineStr"/>
-      <c r="V2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W2" s="7" t="n">
+      <c r="N2" s="9" t="inlineStr"/>
+      <c r="O2" s="9" t="inlineStr"/>
+      <c r="P2" s="9" t="inlineStr"/>
+      <c r="Q2" s="9" t="inlineStr"/>
+      <c r="R2" s="9" t="inlineStr"/>
+      <c r="S2" s="9" t="inlineStr"/>
+      <c r="T2" s="9" t="inlineStr"/>
+      <c r="U2" s="9" t="inlineStr"/>
+      <c r="V2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="W2" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="X2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="Y2" s="7" t="n">
+      <c r="X2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="Y2" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="Z2" s="9" t="inlineStr">
+      <c r="Z2" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="AA2" s="6" t="n">
+      <c r="AA2" s="5" t="n">
         <v>0.061</v>
       </c>
-      <c r="AB2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AC2" s="6" t="n">
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AC2" s="5" t="n">
         <v>0.019</v>
       </c>
-      <c r="AD2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AE2" s="7" t="n">
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AE2" s="6" t="n">
         <v>1.48</v>
       </c>
-      <c r="AF2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AG2" s="6" t="n">
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AG2" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="AH2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AI2" s="8" t="n">
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AI2" s="7" t="n">
         <v>33</v>
       </c>
-      <c r="AJ2" s="9" t="inlineStr">
+      <c r="AJ2" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="AK2" s="8" t="n">
+      <c r="AK2" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="AL2" s="10" t="inlineStr"/>
-      <c r="AM2" s="10" t="inlineStr"/>
-      <c r="AN2" s="10" t="inlineStr"/>
-      <c r="AO2" s="10" t="inlineStr"/>
-      <c r="AP2" s="10" t="inlineStr"/>
-      <c r="AQ2" s="10" t="inlineStr"/>
-      <c r="AR2" s="10" t="inlineStr"/>
-      <c r="AS2" s="10" t="inlineStr"/>
-      <c r="AT2" s="10" t="inlineStr"/>
-      <c r="AU2" s="10" t="inlineStr"/>
-      <c r="AV2" s="10" t="inlineStr"/>
-      <c r="AW2" s="10" t="inlineStr"/>
-      <c r="AX2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AY2" s="6" t="n">
+      <c r="AL2" s="9" t="inlineStr"/>
+      <c r="AM2" s="9" t="inlineStr"/>
+      <c r="AN2" s="9" t="inlineStr"/>
+      <c r="AO2" s="9" t="inlineStr"/>
+      <c r="AP2" s="9" t="inlineStr"/>
+      <c r="AQ2" s="9" t="inlineStr"/>
+      <c r="AR2" s="9" t="inlineStr"/>
+      <c r="AS2" s="9" t="inlineStr"/>
+      <c r="AT2" s="9" t="inlineStr"/>
+      <c r="AU2" s="9" t="inlineStr"/>
+      <c r="AV2" s="9" t="inlineStr"/>
+      <c r="AW2" s="9" t="inlineStr"/>
+      <c r="AX2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AY2" s="5" t="n">
         <v>0.029</v>
       </c>
-      <c r="AZ2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BA2" s="6" t="n">
+      <c r="AZ2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BA2" s="5" t="n">
         <v>0.023</v>
       </c>
-      <c r="BB2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BC2" s="6" t="n">
+      <c r="BB2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BC2" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="BD2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BE2" s="7" t="n">
+      <c r="BD2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BE2" s="6" t="n">
         <v>1.75</v>
       </c>
-      <c r="BF2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BG2" s="8" t="n">
+      <c r="BF2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BG2" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="BH2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BI2" s="8" t="n">
+      <c r="BH2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BI2" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="BJ2" s="11" t="inlineStr">
+      <c r="BJ2" s="10" t="inlineStr">
         <is>
           <t>Muy Mala</t>
         </is>
       </c>
-      <c r="BK2" s="6" t="n">
+      <c r="BK2" s="5" t="n">
         <v>0.144</v>
       </c>
-      <c r="BL2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BM2" s="6" t="n">
+      <c r="BL2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BM2" s="5" t="n">
         <v>0.024</v>
       </c>
-      <c r="BN2" s="10" t="inlineStr"/>
-      <c r="BO2" s="10" t="inlineStr"/>
-      <c r="BP2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BQ2" s="7" t="n">
+      <c r="BN2" s="9" t="inlineStr"/>
+      <c r="BO2" s="9" t="inlineStr"/>
+      <c r="BP2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BQ2" s="6" t="n">
         <v>0.65</v>
       </c>
-      <c r="BR2" s="9" t="inlineStr">
+      <c r="BR2" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="BS2" s="8" t="n">
+      <c r="BS2" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="BT2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BU2" s="8" t="n">
+      <c r="BT2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BU2" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="BV2" s="9" t="inlineStr">
+      <c r="BV2" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="BW2" s="6" t="n">
+      <c r="BW2" s="5" t="n">
         <v>0.061</v>
       </c>
-      <c r="BX2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BY2" s="6" t="n">
+      <c r="BX2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BY2" s="5" t="n">
         <v>0.02</v>
       </c>
-      <c r="BZ2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CA2" s="7" t="n">
+      <c r="BZ2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CA2" s="6" t="n">
         <v>0.65</v>
       </c>
-      <c r="CB2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CC2" s="6" t="n">
+      <c r="CB2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CC2" s="5" t="n">
         <v>0.001</v>
       </c>
-      <c r="CD2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CE2" s="8" t="n">
+      <c r="CD2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CE2" s="7" t="n">
         <v>29</v>
       </c>
-      <c r="CF2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CG2" s="8" t="n">
+      <c r="CF2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CG2" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="CH2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CI2" s="6" t="n">
+      <c r="CH2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CI2" s="5" t="n">
         <v>0.054</v>
       </c>
-      <c r="CJ2" s="10" t="inlineStr"/>
-      <c r="CK2" s="10" t="inlineStr"/>
-      <c r="CL2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CM2" s="7" t="n">
+      <c r="CJ2" s="9" t="inlineStr"/>
+      <c r="CK2" s="9" t="inlineStr"/>
+      <c r="CL2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CM2" s="6" t="n">
         <v>0.68</v>
       </c>
-      <c r="CN2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CO2" s="6" t="n">
+      <c r="CN2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CO2" s="5" t="n">
         <v>0.001</v>
       </c>
-      <c r="CP2" s="12" t="inlineStr">
+      <c r="CP2" s="11" t="inlineStr">
         <is>
           <t>Mala</t>
         </is>
       </c>
-      <c r="CQ2" s="8" t="n">
+      <c r="CQ2" s="7" t="n">
         <v>52</v>
       </c>
-      <c r="CR2" s="10" t="inlineStr"/>
-      <c r="CS2" s="10" t="inlineStr"/>
-      <c r="CT2" s="11" t="inlineStr">
+      <c r="CR2" s="9" t="inlineStr"/>
+      <c r="CS2" s="9" t="inlineStr"/>
+      <c r="CT2" s="10" t="inlineStr">
         <is>
           <t>Muy Mala</t>
         </is>
       </c>
     </row>
     <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="3" t="n">
         <v>46055</v>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="C3" s="5" t="n">
         <v>0.074</v>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="n">
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="n">
         <v>0.022</v>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="n">
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="n">
         <v>0.54</v>
       </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="n">
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="n">
         <v>0.001</v>
       </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="n">
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="L3" s="9" t="inlineStr">
+      <c r="L3" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="M3" s="8" t="n">
+      <c r="M3" s="7" t="n">
         <v>17</v>
       </c>
-      <c r="N3" s="10" t="inlineStr"/>
-      <c r="O3" s="10" t="inlineStr"/>
-      <c r="P3" s="10" t="inlineStr"/>
-      <c r="Q3" s="10" t="inlineStr"/>
-      <c r="R3" s="10" t="inlineStr"/>
-      <c r="S3" s="10" t="inlineStr"/>
-      <c r="T3" s="10" t="inlineStr"/>
-      <c r="U3" s="10" t="inlineStr"/>
-      <c r="V3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="W3" s="7" t="n">
+      <c r="N3" s="9" t="inlineStr"/>
+      <c r="O3" s="9" t="inlineStr"/>
+      <c r="P3" s="9" t="inlineStr"/>
+      <c r="Q3" s="9" t="inlineStr"/>
+      <c r="R3" s="9" t="inlineStr"/>
+      <c r="S3" s="9" t="inlineStr"/>
+      <c r="T3" s="9" t="inlineStr"/>
+      <c r="U3" s="9" t="inlineStr"/>
+      <c r="V3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="W3" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="X3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="Y3" s="7" t="n">
+      <c r="X3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="Y3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="Z3" s="9" t="inlineStr">
+      <c r="Z3" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="AA3" s="6" t="n">
+      <c r="AA3" s="5" t="n">
         <v>0.079</v>
       </c>
-      <c r="AB3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AC3" s="6" t="n">
+      <c r="AB3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AC3" s="5" t="n">
         <v>0.027</v>
       </c>
-      <c r="AD3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AE3" s="7" t="n">
+      <c r="AD3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AE3" s="6" t="n">
         <v>1.52</v>
       </c>
-      <c r="AF3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AG3" s="6" t="n">
+      <c r="AF3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AG3" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="AH3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AI3" s="8" t="n">
+      <c r="AH3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AI3" s="7" t="n">
         <v>34</v>
       </c>
-      <c r="AJ3" s="9" t="inlineStr">
+      <c r="AJ3" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="AK3" s="8" t="n">
+      <c r="AK3" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="AL3" s="10" t="inlineStr"/>
-      <c r="AM3" s="10" t="inlineStr"/>
-      <c r="AN3" s="10" t="inlineStr"/>
-      <c r="AO3" s="10" t="inlineStr"/>
-      <c r="AP3" s="10" t="inlineStr"/>
-      <c r="AQ3" s="10" t="inlineStr"/>
-      <c r="AR3" s="10" t="inlineStr"/>
-      <c r="AS3" s="10" t="inlineStr"/>
-      <c r="AT3" s="10" t="inlineStr"/>
-      <c r="AU3" s="10" t="inlineStr"/>
-      <c r="AV3" s="10" t="inlineStr"/>
-      <c r="AW3" s="10" t="inlineStr"/>
-      <c r="AX3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AY3" s="6" t="n">
+      <c r="AL3" s="9" t="inlineStr"/>
+      <c r="AM3" s="9" t="inlineStr"/>
+      <c r="AN3" s="9" t="inlineStr"/>
+      <c r="AO3" s="9" t="inlineStr"/>
+      <c r="AP3" s="9" t="inlineStr"/>
+      <c r="AQ3" s="9" t="inlineStr"/>
+      <c r="AR3" s="9" t="inlineStr"/>
+      <c r="AS3" s="9" t="inlineStr"/>
+      <c r="AT3" s="9" t="inlineStr"/>
+      <c r="AU3" s="9" t="inlineStr"/>
+      <c r="AV3" s="9" t="inlineStr"/>
+      <c r="AW3" s="9" t="inlineStr"/>
+      <c r="AX3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AY3" s="5" t="n">
         <v>0.025</v>
       </c>
-      <c r="AZ3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BA3" s="6" t="n">
+      <c r="AZ3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BA3" s="5" t="n">
         <v>0.036</v>
       </c>
-      <c r="BB3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BC3" s="6" t="n">
+      <c r="BB3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BC3" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="BD3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BE3" s="7" t="n">
+      <c r="BD3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BE3" s="6" t="n">
         <v>1.85</v>
       </c>
-      <c r="BF3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BG3" s="8" t="n">
+      <c r="BF3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BG3" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="BH3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BI3" s="8" t="n">
+      <c r="BH3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BI3" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="BJ3" s="9" t="inlineStr">
+      <c r="BJ3" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="BK3" s="6" t="n">
+      <c r="BK3" s="5" t="n">
         <v>0.066</v>
       </c>
-      <c r="BL3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BM3" s="6" t="n">
+      <c r="BL3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BM3" s="5" t="n">
         <v>0.032</v>
       </c>
-      <c r="BN3" s="10" t="inlineStr"/>
-      <c r="BO3" s="10" t="inlineStr"/>
-      <c r="BP3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BQ3" s="7" t="n">
+      <c r="BN3" s="9" t="inlineStr"/>
+      <c r="BO3" s="9" t="inlineStr"/>
+      <c r="BP3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BQ3" s="6" t="n">
         <v>0.73</v>
       </c>
-      <c r="BR3" s="9" t="inlineStr">
+      <c r="BR3" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="BS3" s="8" t="n">
+      <c r="BS3" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="BT3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BU3" s="8" t="n">
+      <c r="BT3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BU3" s="7" t="n">
         <v>43</v>
       </c>
-      <c r="BV3" s="9" t="inlineStr">
+      <c r="BV3" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="BW3" s="6" t="n">
+      <c r="BW3" s="5" t="n">
         <v>0.073</v>
       </c>
-      <c r="BX3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BY3" s="6" t="n">
+      <c r="BX3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BY3" s="5" t="n">
         <v>0.022</v>
       </c>
-      <c r="BZ3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CA3" s="7" t="n">
+      <c r="BZ3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CA3" s="6" t="n">
         <v>0.73</v>
       </c>
-      <c r="CB3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CC3" s="6" t="n">
+      <c r="CB3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CC3" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="CD3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CE3" s="8" t="n">
+      <c r="CD3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CE3" s="7" t="n">
         <v>31</v>
       </c>
-      <c r="CF3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CG3" s="8" t="n">
+      <c r="CF3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CG3" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="CH3" s="9" t="inlineStr">
+      <c r="CH3" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="CI3" s="6" t="n">
+      <c r="CI3" s="5" t="n">
         <v>0.063</v>
       </c>
-      <c r="CJ3" s="10" t="inlineStr"/>
-      <c r="CK3" s="10" t="inlineStr"/>
-      <c r="CL3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CM3" s="7" t="n">
+      <c r="CJ3" s="9" t="inlineStr"/>
+      <c r="CK3" s="9" t="inlineStr"/>
+      <c r="CL3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CM3" s="6" t="n">
         <v>0.78</v>
       </c>
-      <c r="CN3" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CO3" s="6" t="n">
+      <c r="CN3" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CO3" s="5" t="n">
         <v>0.001</v>
       </c>
-      <c r="CP3" s="12" t="inlineStr">
+      <c r="CP3" s="11" t="inlineStr">
         <is>
           <t>Mala</t>
         </is>
       </c>
-      <c r="CQ3" s="8" t="n">
+      <c r="CQ3" s="7" t="n">
         <v>58</v>
       </c>
-      <c r="CR3" s="10" t="inlineStr"/>
-      <c r="CS3" s="10" t="inlineStr"/>
-      <c r="CT3" s="12" t="inlineStr">
+      <c r="CR3" s="9" t="inlineStr"/>
+      <c r="CS3" s="9" t="inlineStr"/>
+      <c r="CT3" s="11" t="inlineStr">
         <is>
           <t>Mala</t>
         </is>
       </c>
     </row>
     <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="3" t="n">
         <v>46056</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="n">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
         <v>0.047</v>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="n">
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="n">
         <v>0.026</v>
       </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="n">
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="n">
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="n">
         <v>0.003</v>
       </c>
-      <c r="J4" s="10" t="inlineStr"/>
-      <c r="K4" s="10" t="inlineStr"/>
-      <c r="L4" s="10" t="inlineStr"/>
-      <c r="M4" s="10" t="inlineStr"/>
-      <c r="N4" s="10" t="inlineStr"/>
-      <c r="O4" s="10" t="inlineStr"/>
-      <c r="P4" s="10" t="inlineStr"/>
-      <c r="Q4" s="10" t="inlineStr"/>
-      <c r="R4" s="10" t="inlineStr"/>
-      <c r="S4" s="10" t="inlineStr"/>
-      <c r="T4" s="10" t="inlineStr"/>
-      <c r="U4" s="10" t="inlineStr"/>
-      <c r="V4" s="10" t="inlineStr"/>
-      <c r="W4" s="10" t="inlineStr"/>
-      <c r="X4" s="10" t="inlineStr"/>
-      <c r="Y4" s="10" t="inlineStr"/>
-      <c r="Z4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AA4" s="6" t="n">
+      <c r="J4" s="9" t="inlineStr"/>
+      <c r="K4" s="9" t="inlineStr"/>
+      <c r="L4" s="9" t="inlineStr"/>
+      <c r="M4" s="9" t="inlineStr"/>
+      <c r="N4" s="9" t="inlineStr"/>
+      <c r="O4" s="9" t="inlineStr"/>
+      <c r="P4" s="9" t="inlineStr"/>
+      <c r="Q4" s="9" t="inlineStr"/>
+      <c r="R4" s="9" t="inlineStr"/>
+      <c r="S4" s="9" t="inlineStr"/>
+      <c r="T4" s="9" t="inlineStr"/>
+      <c r="U4" s="9" t="inlineStr"/>
+      <c r="V4" s="9" t="inlineStr"/>
+      <c r="W4" s="9" t="inlineStr"/>
+      <c r="X4" s="9" t="inlineStr"/>
+      <c r="Y4" s="9" t="inlineStr"/>
+      <c r="Z4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AA4" s="5" t="n">
         <v>0.043</v>
       </c>
-      <c r="AB4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AC4" s="6" t="n">
+      <c r="AB4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AC4" s="5" t="n">
         <v>0.029</v>
       </c>
-      <c r="AD4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AE4" s="7" t="n">
+      <c r="AD4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AE4" s="6" t="n">
         <v>1.6</v>
       </c>
-      <c r="AF4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AG4" s="6" t="n">
+      <c r="AF4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AG4" s="5" t="n">
         <v>0.003</v>
       </c>
-      <c r="AH4" s="10" t="inlineStr"/>
-      <c r="AI4" s="10" t="inlineStr"/>
-      <c r="AJ4" s="10" t="inlineStr"/>
-      <c r="AK4" s="10" t="inlineStr"/>
-      <c r="AL4" s="10" t="inlineStr"/>
-      <c r="AM4" s="10" t="inlineStr"/>
-      <c r="AN4" s="10" t="inlineStr"/>
-      <c r="AO4" s="10" t="inlineStr"/>
-      <c r="AP4" s="10" t="inlineStr"/>
-      <c r="AQ4" s="10" t="inlineStr"/>
-      <c r="AR4" s="10" t="inlineStr"/>
-      <c r="AS4" s="10" t="inlineStr"/>
-      <c r="AT4" s="10" t="inlineStr"/>
-      <c r="AU4" s="10" t="inlineStr"/>
-      <c r="AV4" s="10" t="inlineStr"/>
-      <c r="AW4" s="10" t="inlineStr"/>
-      <c r="AX4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AY4" s="6" t="n">
+      <c r="AH4" s="9" t="inlineStr"/>
+      <c r="AI4" s="9" t="inlineStr"/>
+      <c r="AJ4" s="9" t="inlineStr"/>
+      <c r="AK4" s="9" t="inlineStr"/>
+      <c r="AL4" s="9" t="inlineStr"/>
+      <c r="AM4" s="9" t="inlineStr"/>
+      <c r="AN4" s="9" t="inlineStr"/>
+      <c r="AO4" s="9" t="inlineStr"/>
+      <c r="AP4" s="9" t="inlineStr"/>
+      <c r="AQ4" s="9" t="inlineStr"/>
+      <c r="AR4" s="9" t="inlineStr"/>
+      <c r="AS4" s="9" t="inlineStr"/>
+      <c r="AT4" s="9" t="inlineStr"/>
+      <c r="AU4" s="9" t="inlineStr"/>
+      <c r="AV4" s="9" t="inlineStr"/>
+      <c r="AW4" s="9" t="inlineStr"/>
+      <c r="AX4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AY4" s="5" t="n">
         <v>0.022</v>
       </c>
-      <c r="AZ4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BA4" s="6" t="n">
+      <c r="AZ4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BA4" s="5" t="n">
         <v>0.029</v>
       </c>
-      <c r="BB4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BC4" s="6" t="n">
+      <c r="BB4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BC4" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="BD4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BE4" s="7" t="n">
+      <c r="BD4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BE4" s="6" t="n">
         <v>1.95</v>
       </c>
-      <c r="BF4" s="10" t="inlineStr"/>
-      <c r="BG4" s="10" t="inlineStr"/>
-      <c r="BH4" s="10" t="inlineStr"/>
-      <c r="BI4" s="10" t="inlineStr"/>
-      <c r="BJ4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BK4" s="6" t="n">
+      <c r="BF4" s="9" t="inlineStr"/>
+      <c r="BG4" s="9" t="inlineStr"/>
+      <c r="BH4" s="9" t="inlineStr"/>
+      <c r="BI4" s="9" t="inlineStr"/>
+      <c r="BJ4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BK4" s="5" t="n">
         <v>0.043</v>
       </c>
-      <c r="BL4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BM4" s="6" t="n">
+      <c r="BL4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BM4" s="5" t="n">
         <v>0.023</v>
       </c>
-      <c r="BN4" s="10" t="inlineStr"/>
-      <c r="BO4" s="10" t="inlineStr"/>
-      <c r="BP4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BQ4" s="7" t="n">
+      <c r="BN4" s="9" t="inlineStr"/>
+      <c r="BO4" s="9" t="inlineStr"/>
+      <c r="BP4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BQ4" s="6" t="n">
         <v>0.75</v>
       </c>
-      <c r="BR4" s="10" t="inlineStr"/>
-      <c r="BS4" s="10" t="inlineStr"/>
-      <c r="BT4" s="10" t="inlineStr"/>
-      <c r="BU4" s="10" t="inlineStr"/>
-      <c r="BV4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BW4" s="6" t="n">
+      <c r="BR4" s="9" t="inlineStr"/>
+      <c r="BS4" s="9" t="inlineStr"/>
+      <c r="BT4" s="9" t="inlineStr"/>
+      <c r="BU4" s="9" t="inlineStr"/>
+      <c r="BV4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BW4" s="5" t="n">
         <v>0.052</v>
       </c>
-      <c r="BX4" s="9" t="inlineStr">
+      <c r="BX4" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="BY4" s="6" t="n">
+      <c r="BY4" s="5" t="n">
         <v>0.066</v>
       </c>
-      <c r="BZ4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CA4" s="7" t="n">
+      <c r="BZ4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CA4" s="6" t="n">
         <v>1.56</v>
       </c>
-      <c r="CB4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CC4" s="6" t="n">
+      <c r="CB4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CC4" s="5" t="n">
         <v>0.003</v>
       </c>
-      <c r="CD4" s="10" t="inlineStr"/>
-      <c r="CE4" s="10" t="inlineStr"/>
-      <c r="CF4" s="10" t="inlineStr"/>
-      <c r="CG4" s="10" t="inlineStr"/>
-      <c r="CH4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CI4" s="6" t="n">
+      <c r="CD4" s="9" t="inlineStr"/>
+      <c r="CE4" s="9" t="inlineStr"/>
+      <c r="CF4" s="9" t="inlineStr"/>
+      <c r="CG4" s="9" t="inlineStr"/>
+      <c r="CH4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CI4" s="5" t="n">
         <v>0.034</v>
       </c>
-      <c r="CJ4" s="10" t="inlineStr"/>
-      <c r="CK4" s="10" t="inlineStr"/>
-      <c r="CL4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CM4" s="7" t="n">
+      <c r="CJ4" s="9" t="inlineStr"/>
+      <c r="CK4" s="9" t="inlineStr"/>
+      <c r="CL4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CM4" s="6" t="n">
         <v>1.19</v>
       </c>
-      <c r="CN4" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CO4" s="6" t="n">
+      <c r="CN4" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CO4" s="5" t="n">
         <v>0.001</v>
       </c>
-      <c r="CP4" s="10" t="inlineStr"/>
-      <c r="CQ4" s="10" t="inlineStr"/>
-      <c r="CR4" s="10" t="inlineStr"/>
-      <c r="CS4" s="10" t="inlineStr"/>
-      <c r="CT4" s="9" t="inlineStr">
+      <c r="CP4" s="9" t="inlineStr"/>
+      <c r="CQ4" s="9" t="inlineStr"/>
+      <c r="CR4" s="9" t="inlineStr"/>
+      <c r="CS4" s="9" t="inlineStr"/>
+      <c r="CT4" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
@@ -2072,694 +2063,694 @@
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_AGUA SANTA</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_AGUA SANTA</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_AGUA SANTA</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_AGUA SANTA</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_AGUA SANTA</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_AGUA SANTA</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_AGUA SANTA</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_AGUA SANTA</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_AGUA SANTA</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_AGUA SANTA</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_AGUA SANTA</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_AGUA SANTA</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_ATLIXCO</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_ATLIXCO</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_ATLIXCO</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_ATLIXCO</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_ATLIXCO</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_ATLIXCO</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_ATLIXCO</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_ATLIXCO</t>
         </is>
       </c>
-      <c r="V1" s="3" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_ATLIXCO</t>
         </is>
       </c>
-      <c r="W1" s="3" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_ATLIXCO</t>
         </is>
       </c>
-      <c r="X1" s="3" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_ATLIXCO</t>
         </is>
       </c>
-      <c r="Y1" s="3" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_ATLIXCO</t>
         </is>
       </c>
-      <c r="Z1" s="3" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_BINE</t>
         </is>
       </c>
-      <c r="AA1" s="3" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_BINE</t>
         </is>
       </c>
-      <c r="AB1" s="3" t="inlineStr">
+      <c r="AB1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_BINE</t>
         </is>
       </c>
-      <c r="AC1" s="3" t="inlineStr">
+      <c r="AC1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_BINE</t>
         </is>
       </c>
-      <c r="AD1" s="3" t="inlineStr">
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_BINE</t>
         </is>
       </c>
-      <c r="AE1" s="3" t="inlineStr">
+      <c r="AE1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_BINE</t>
         </is>
       </c>
-      <c r="AF1" s="3" t="inlineStr">
+      <c r="AF1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_BINE</t>
         </is>
       </c>
-      <c r="AG1" s="3" t="inlineStr">
+      <c r="AG1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_BINE</t>
         </is>
       </c>
-      <c r="AH1" s="3" t="inlineStr">
+      <c r="AH1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_BINE</t>
         </is>
       </c>
-      <c r="AI1" s="3" t="inlineStr">
+      <c r="AI1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_BINE</t>
         </is>
       </c>
-      <c r="AJ1" s="3" t="inlineStr">
+      <c r="AJ1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_BINE</t>
         </is>
       </c>
-      <c r="AK1" s="3" t="inlineStr">
+      <c r="AK1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_BINE</t>
         </is>
       </c>
-      <c r="AL1" s="3" t="inlineStr">
+      <c r="AL1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_NINFAS</t>
         </is>
       </c>
-      <c r="AM1" s="3" t="inlineStr">
+      <c r="AM1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_NINFAS</t>
         </is>
       </c>
-      <c r="AN1" s="3" t="inlineStr">
+      <c r="AN1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_NINFAS</t>
         </is>
       </c>
-      <c r="AO1" s="3" t="inlineStr">
+      <c r="AO1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_NINFAS</t>
         </is>
       </c>
-      <c r="AP1" s="3" t="inlineStr">
+      <c r="AP1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_NINFAS</t>
         </is>
       </c>
-      <c r="AQ1" s="3" t="inlineStr">
+      <c r="AQ1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_NINFAS</t>
         </is>
       </c>
-      <c r="AR1" s="3" t="inlineStr">
+      <c r="AR1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_NINFAS</t>
         </is>
       </c>
-      <c r="AS1" s="3" t="inlineStr">
+      <c r="AS1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_NINFAS</t>
         </is>
       </c>
-      <c r="AT1" s="3" t="inlineStr">
+      <c r="AT1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_NINFAS</t>
         </is>
       </c>
-      <c r="AU1" s="3" t="inlineStr">
+      <c r="AU1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_NINFAS</t>
         </is>
       </c>
-      <c r="AV1" s="3" t="inlineStr">
+      <c r="AV1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_NINFAS</t>
         </is>
       </c>
-      <c r="AW1" s="3" t="inlineStr">
+      <c r="AW1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_NINFAS</t>
         </is>
       </c>
-      <c r="AX1" s="3" t="inlineStr">
+      <c r="AX1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_TEHUACAN</t>
         </is>
       </c>
-      <c r="AY1" s="3" t="inlineStr">
+      <c r="AY1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_TEHUACAN</t>
         </is>
       </c>
-      <c r="AZ1" s="3" t="inlineStr">
+      <c r="AZ1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_TEHUACAN</t>
         </is>
       </c>
-      <c r="BA1" s="3" t="inlineStr">
+      <c r="BA1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_TEHUACAN</t>
         </is>
       </c>
-      <c r="BB1" s="3" t="inlineStr">
+      <c r="BB1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_TEHUACAN</t>
         </is>
       </c>
-      <c r="BC1" s="3" t="inlineStr">
+      <c r="BC1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_TEHUACAN</t>
         </is>
       </c>
-      <c r="BD1" s="3" t="inlineStr">
+      <c r="BD1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_TEHUACAN</t>
         </is>
       </c>
-      <c r="BE1" s="3" t="inlineStr">
+      <c r="BE1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_TEHUACAN</t>
         </is>
       </c>
-      <c r="BF1" s="3" t="inlineStr">
+      <c r="BF1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_TEHUACAN</t>
         </is>
       </c>
-      <c r="BG1" s="3" t="inlineStr">
+      <c r="BG1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_TEHUACAN</t>
         </is>
       </c>
-      <c r="BH1" s="3" t="inlineStr">
+      <c r="BH1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_TEHUACAN</t>
         </is>
       </c>
-      <c r="BI1" s="3" t="inlineStr">
+      <c r="BI1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_TEHUACAN</t>
         </is>
       </c>
-      <c r="BJ1" s="3" t="inlineStr">
+      <c r="BJ1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BK1" s="3" t="inlineStr">
+      <c r="BK1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BL1" s="3" t="inlineStr">
+      <c r="BL1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BM1" s="3" t="inlineStr">
+      <c r="BM1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BN1" s="3" t="inlineStr">
+      <c r="BN1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BO1" s="3" t="inlineStr">
+      <c r="BO1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BP1" s="3" t="inlineStr">
+      <c r="BP1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BQ1" s="3" t="inlineStr">
+      <c r="BQ1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BR1" s="3" t="inlineStr">
+      <c r="BR1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BS1" s="3" t="inlineStr">
+      <c r="BS1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BT1" s="3" t="inlineStr">
+      <c r="BT1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BU1" s="3" t="inlineStr">
+      <c r="BU1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_TEXMELUCAN</t>
         </is>
       </c>
-      <c r="BV1" s="3" t="inlineStr">
+      <c r="BV1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_UTP</t>
         </is>
       </c>
-      <c r="BW1" s="3" t="inlineStr">
+      <c r="BW1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_UTP</t>
         </is>
       </c>
-      <c r="BX1" s="3" t="inlineStr">
+      <c r="BX1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_UTP</t>
         </is>
       </c>
-      <c r="BY1" s="3" t="inlineStr">
+      <c r="BY1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_UTP</t>
         </is>
       </c>
-      <c r="BZ1" s="3" t="inlineStr">
+      <c r="BZ1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_UTP</t>
         </is>
       </c>
-      <c r="CA1" s="3" t="inlineStr">
+      <c r="CA1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_UTP</t>
         </is>
       </c>
-      <c r="CB1" s="3" t="inlineStr">
+      <c r="CB1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_UTP</t>
         </is>
       </c>
-      <c r="CC1" s="3" t="inlineStr">
+      <c r="CC1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_UTP</t>
         </is>
       </c>
-      <c r="CD1" s="3" t="inlineStr">
+      <c r="CD1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_UTP</t>
         </is>
       </c>
-      <c r="CE1" s="3" t="inlineStr">
+      <c r="CE1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_UTP</t>
         </is>
       </c>
-      <c r="CF1" s="3" t="inlineStr">
+      <c r="CF1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_UTP</t>
         </is>
       </c>
-      <c r="CG1" s="3" t="inlineStr">
+      <c r="CG1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_UTP</t>
         </is>
       </c>
-      <c r="CH1" s="3" t="inlineStr">
+      <c r="CH1" s="2" t="inlineStr">
         <is>
           <t>AIRE_O3_VELODROMO</t>
         </is>
       </c>
-      <c r="CI1" s="3" t="inlineStr">
+      <c r="CI1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_O3_VELODROMO</t>
         </is>
       </c>
-      <c r="CJ1" s="3" t="inlineStr">
+      <c r="CJ1" s="2" t="inlineStr">
         <is>
           <t>AIRE_NO2_VELODROMO</t>
         </is>
       </c>
-      <c r="CK1" s="3" t="inlineStr">
+      <c r="CK1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_NO2_VELODROMO</t>
         </is>
       </c>
-      <c r="CL1" s="3" t="inlineStr">
+      <c r="CL1" s="2" t="inlineStr">
         <is>
           <t>AIRE_CO_VELODROMO</t>
         </is>
       </c>
-      <c r="CM1" s="3" t="inlineStr">
+      <c r="CM1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_CO_VELODROMO</t>
         </is>
       </c>
-      <c r="CN1" s="3" t="inlineStr">
+      <c r="CN1" s="2" t="inlineStr">
         <is>
           <t>AIRE_SO2_VELODROMO</t>
         </is>
       </c>
-      <c r="CO1" s="3" t="inlineStr">
+      <c r="CO1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_SO2_VELODROMO</t>
         </is>
       </c>
-      <c r="CP1" s="3" t="inlineStr">
+      <c r="CP1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM10_VELODROMO</t>
         </is>
       </c>
-      <c r="CQ1" s="3" t="inlineStr">
+      <c r="CQ1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM10_VELODROMO</t>
         </is>
       </c>
-      <c r="CR1" s="3" t="inlineStr">
+      <c r="CR1" s="2" t="inlineStr">
         <is>
           <t>AIRE_PM2.5_VELODROMO</t>
         </is>
       </c>
-      <c r="CS1" s="3" t="inlineStr">
+      <c r="CS1" s="2" t="inlineStr">
         <is>
           <t>CANTIDAD_PM2.5_VELODROMO</t>
         </is>
       </c>
-      <c r="CT1" s="3" t="inlineStr">
+      <c r="CT1" s="2" t="inlineStr">
         <is>
           <t>Calidad del aire</t>
         </is>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="4" t="n">
+      <c r="A2" s="3" t="n">
         <v>46056</v>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="C2" s="6" t="n">
+      <c r="C2" s="5" t="n">
         <v>0.078</v>
       </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="n">
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n">
         <v>0.008</v>
       </c>
-      <c r="F2" s="10" t="inlineStr"/>
-      <c r="G2" s="10" t="inlineStr"/>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="n">
+      <c r="F2" s="9" t="inlineStr"/>
+      <c r="G2" s="9" t="inlineStr"/>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="J2" s="10" t="inlineStr"/>
-      <c r="K2" s="10" t="inlineStr"/>
-      <c r="L2" s="10" t="inlineStr"/>
-      <c r="M2" s="10" t="inlineStr"/>
-      <c r="N2" s="10" t="inlineStr"/>
-      <c r="O2" s="10" t="inlineStr"/>
-      <c r="P2" s="10" t="inlineStr"/>
-      <c r="Q2" s="10" t="inlineStr"/>
-      <c r="R2" s="10" t="inlineStr"/>
-      <c r="S2" s="10" t="inlineStr"/>
-      <c r="T2" s="10" t="inlineStr"/>
-      <c r="U2" s="10" t="inlineStr"/>
-      <c r="V2" s="10" t="inlineStr"/>
-      <c r="W2" s="10" t="inlineStr"/>
-      <c r="X2" s="10" t="inlineStr"/>
-      <c r="Y2" s="10" t="inlineStr"/>
-      <c r="Z2" s="9" t="inlineStr">
+      <c r="J2" s="9" t="inlineStr"/>
+      <c r="K2" s="9" t="inlineStr"/>
+      <c r="L2" s="9" t="inlineStr"/>
+      <c r="M2" s="9" t="inlineStr"/>
+      <c r="N2" s="9" t="inlineStr"/>
+      <c r="O2" s="9" t="inlineStr"/>
+      <c r="P2" s="9" t="inlineStr"/>
+      <c r="Q2" s="9" t="inlineStr"/>
+      <c r="R2" s="9" t="inlineStr"/>
+      <c r="S2" s="9" t="inlineStr"/>
+      <c r="T2" s="9" t="inlineStr"/>
+      <c r="U2" s="9" t="inlineStr"/>
+      <c r="V2" s="9" t="inlineStr"/>
+      <c r="W2" s="9" t="inlineStr"/>
+      <c r="X2" s="9" t="inlineStr"/>
+      <c r="Y2" s="9" t="inlineStr"/>
+      <c r="Z2" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="AA2" s="6" t="n">
+      <c r="AA2" s="5" t="n">
         <v>0.08</v>
       </c>
-      <c r="AB2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AC2" s="6" t="n">
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AC2" s="5" t="n">
         <v>0.012</v>
       </c>
-      <c r="AD2" s="10" t="inlineStr"/>
-      <c r="AE2" s="10" t="inlineStr"/>
-      <c r="AF2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AG2" s="6" t="n">
+      <c r="AD2" s="9" t="inlineStr"/>
+      <c r="AE2" s="9" t="inlineStr"/>
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AG2" s="5" t="n">
         <v>0.001</v>
       </c>
-      <c r="AH2" s="10" t="inlineStr"/>
-      <c r="AI2" s="10" t="inlineStr"/>
-      <c r="AJ2" s="10" t="inlineStr"/>
-      <c r="AK2" s="10" t="inlineStr"/>
-      <c r="AL2" s="10" t="inlineStr"/>
-      <c r="AM2" s="10" t="inlineStr"/>
-      <c r="AN2" s="10" t="inlineStr"/>
-      <c r="AO2" s="10" t="inlineStr"/>
-      <c r="AP2" s="10" t="inlineStr"/>
-      <c r="AQ2" s="10" t="inlineStr"/>
-      <c r="AR2" s="10" t="inlineStr"/>
-      <c r="AS2" s="10" t="inlineStr"/>
-      <c r="AT2" s="10" t="inlineStr"/>
-      <c r="AU2" s="10" t="inlineStr"/>
-      <c r="AV2" s="10" t="inlineStr"/>
-      <c r="AW2" s="10" t="inlineStr"/>
-      <c r="AX2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="AY2" s="6" t="n">
+      <c r="AH2" s="9" t="inlineStr"/>
+      <c r="AI2" s="9" t="inlineStr"/>
+      <c r="AJ2" s="9" t="inlineStr"/>
+      <c r="AK2" s="9" t="inlineStr"/>
+      <c r="AL2" s="9" t="inlineStr"/>
+      <c r="AM2" s="9" t="inlineStr"/>
+      <c r="AN2" s="9" t="inlineStr"/>
+      <c r="AO2" s="9" t="inlineStr"/>
+      <c r="AP2" s="9" t="inlineStr"/>
+      <c r="AQ2" s="9" t="inlineStr"/>
+      <c r="AR2" s="9" t="inlineStr"/>
+      <c r="AS2" s="9" t="inlineStr"/>
+      <c r="AT2" s="9" t="inlineStr"/>
+      <c r="AU2" s="9" t="inlineStr"/>
+      <c r="AV2" s="9" t="inlineStr"/>
+      <c r="AW2" s="9" t="inlineStr"/>
+      <c r="AX2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="AY2" s="5" t="n">
         <v>0.029</v>
       </c>
-      <c r="AZ2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BA2" s="6" t="n">
+      <c r="AZ2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BA2" s="5" t="n">
         <v>0.017</v>
       </c>
-      <c r="BB2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BC2" s="6" t="n">
+      <c r="BB2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BC2" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="BD2" s="10" t="inlineStr"/>
-      <c r="BE2" s="10" t="inlineStr"/>
-      <c r="BF2" s="10" t="inlineStr"/>
-      <c r="BG2" s="10" t="inlineStr"/>
-      <c r="BH2" s="10" t="inlineStr"/>
-      <c r="BI2" s="10" t="inlineStr"/>
-      <c r="BJ2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BK2" s="6" t="n">
+      <c r="BD2" s="9" t="inlineStr"/>
+      <c r="BE2" s="9" t="inlineStr"/>
+      <c r="BF2" s="9" t="inlineStr"/>
+      <c r="BG2" s="9" t="inlineStr"/>
+      <c r="BH2" s="9" t="inlineStr"/>
+      <c r="BI2" s="9" t="inlineStr"/>
+      <c r="BJ2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BK2" s="5" t="n">
         <v>0.05</v>
       </c>
-      <c r="BL2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BM2" s="6" t="n">
+      <c r="BL2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BM2" s="5" t="n">
         <v>0.006</v>
       </c>
-      <c r="BN2" s="10" t="inlineStr"/>
-      <c r="BO2" s="10" t="inlineStr"/>
-      <c r="BP2" s="10" t="inlineStr"/>
-      <c r="BQ2" s="10" t="inlineStr"/>
-      <c r="BR2" s="10" t="inlineStr"/>
-      <c r="BS2" s="10" t="inlineStr"/>
-      <c r="BT2" s="10" t="inlineStr"/>
-      <c r="BU2" s="10" t="inlineStr"/>
-      <c r="BV2" s="9" t="inlineStr">
+      <c r="BN2" s="9" t="inlineStr"/>
+      <c r="BO2" s="9" t="inlineStr"/>
+      <c r="BP2" s="9" t="inlineStr"/>
+      <c r="BQ2" s="9" t="inlineStr"/>
+      <c r="BR2" s="9" t="inlineStr"/>
+      <c r="BS2" s="9" t="inlineStr"/>
+      <c r="BT2" s="9" t="inlineStr"/>
+      <c r="BU2" s="9" t="inlineStr"/>
+      <c r="BV2" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="BW2" s="6" t="n">
+      <c r="BW2" s="5" t="n">
         <v>0.076</v>
       </c>
-      <c r="BX2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="BY2" s="6" t="n">
+      <c r="BX2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="BY2" s="5" t="n">
         <v>0.011</v>
       </c>
-      <c r="BZ2" s="10" t="inlineStr"/>
-      <c r="CA2" s="10" t="inlineStr"/>
-      <c r="CB2" s="9" t="inlineStr">
+      <c r="BZ2" s="9" t="inlineStr"/>
+      <c r="CA2" s="9" t="inlineStr"/>
+      <c r="CB2" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="CC2" s="6" t="n">
+      <c r="CC2" s="5" t="n">
         <v>0.058</v>
       </c>
-      <c r="CD2" s="10" t="inlineStr"/>
-      <c r="CE2" s="10" t="inlineStr"/>
-      <c r="CF2" s="10" t="inlineStr"/>
-      <c r="CG2" s="10" t="inlineStr"/>
-      <c r="CH2" s="9" t="inlineStr">
+      <c r="CD2" s="9" t="inlineStr"/>
+      <c r="CE2" s="9" t="inlineStr"/>
+      <c r="CF2" s="9" t="inlineStr"/>
+      <c r="CG2" s="9" t="inlineStr"/>
+      <c r="CH2" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>
       </c>
-      <c r="CI2" s="6" t="n">
+      <c r="CI2" s="5" t="n">
         <v>0.063</v>
       </c>
-      <c r="CJ2" s="10" t="inlineStr"/>
-      <c r="CK2" s="10" t="inlineStr"/>
-      <c r="CL2" s="10" t="inlineStr"/>
-      <c r="CM2" s="10" t="inlineStr"/>
-      <c r="CN2" s="5" t="inlineStr">
-        <is>
-          <t>Buena</t>
-        </is>
-      </c>
-      <c r="CO2" s="6" t="n">
+      <c r="CJ2" s="9" t="inlineStr"/>
+      <c r="CK2" s="9" t="inlineStr"/>
+      <c r="CL2" s="9" t="inlineStr"/>
+      <c r="CM2" s="9" t="inlineStr"/>
+      <c r="CN2" s="4" t="inlineStr">
+        <is>
+          <t>Buena</t>
+        </is>
+      </c>
+      <c r="CO2" s="5" t="n">
         <v>0.001</v>
       </c>
-      <c r="CP2" s="10" t="inlineStr"/>
-      <c r="CQ2" s="10" t="inlineStr"/>
-      <c r="CR2" s="10" t="inlineStr"/>
-      <c r="CS2" s="10" t="inlineStr"/>
-      <c r="CT2" s="9" t="inlineStr">
+      <c r="CP2" s="9" t="inlineStr"/>
+      <c r="CQ2" s="9" t="inlineStr"/>
+      <c r="CR2" s="9" t="inlineStr"/>
+      <c r="CS2" s="9" t="inlineStr"/>
+      <c r="CT2" s="8" t="inlineStr">
         <is>
           <t>Aceptable</t>
         </is>

</xml_diff>